<commit_message>
doing some extra geocoding work
</commit_message>
<xml_diff>
--- a/Sand Project/mine_locs_2024.xlsx
+++ b/Sand Project/mine_locs_2024.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jleedy\Documents\Coursework\SP26\Data Science\solar-incentive-adoption\Sand Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A919073E-54E8-4CEA-BBBB-0B393DB415E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{553D60BE-05B5-4A3A-A10E-380E6A144281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -237,7 +237,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="270">
   <si>
     <t xml:space="preserve"> 59 Federal Road Map 131 Lot 1-1 + 131-1-2 </t>
   </si>
@@ -739,33 +739,18 @@
     <t>Squirrel Island Road</t>
   </si>
   <si>
-    <t>Commerce Park/0 Colony Place  Lot 26</t>
-  </si>
-  <si>
     <t>Colony Place Development LLC</t>
   </si>
   <si>
     <t>Business Park</t>
   </si>
   <si>
-    <t>Commerce Park/ 0 Colony Place Lot 29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commerce Park/Colony Place Map 102/Lot 26-2 </t>
-  </si>
-  <si>
     <t>Gary Darmin</t>
   </si>
   <si>
-    <t xml:space="preserve">Commerce Park Colony Place Map 105, Lot 27 </t>
-  </si>
-  <si>
     <t>Commerce Park LLC</t>
   </si>
   <si>
-    <t xml:space="preserve">Commerce Park Colony Place Map 104 Lot 14  </t>
-  </si>
-  <si>
     <t>Dundee Corp.</t>
   </si>
   <si>
@@ -782,9 +767,6 @@
   </si>
   <si>
     <t>Development</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 360 Cherry Street</t>
   </si>
   <si>
     <t>T.L. Edwards Inc.</t>
@@ -1241,6 +1223,15 @@
   </si>
   <si>
     <t>Park Avenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 360 Cherry Street, Plymouth, MA</t>
+  </si>
+  <si>
+    <t>Commerce Park Colony Place</t>
   </si>
 </sst>
 </file>
@@ -1854,40 +1845,40 @@
   <sheetData>
     <row r="1" spans="1:12" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="G1" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="H1" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="I1" s="7" t="s">
         <v>248</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="J1" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="K1" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="L1" s="6" t="s">
         <v>251</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>253</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -2081,7 +2072,7 @@
     </row>
     <row r="7" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="17" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>1</v>
@@ -2644,7 +2635,7 @@
         <v>52</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="C24" s="15">
         <v>50000</v>
@@ -2682,7 +2673,7 @@
         <v>53</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="C25" s="15">
         <v>2250000</v>
@@ -2718,7 +2709,7 @@
         <v>54</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="C26" s="15">
         <v>60000</v>
@@ -2754,7 +2745,7 @@
         <v>55</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="C27" s="15">
         <v>350000</v>
@@ -3033,7 +3024,7 @@
     </row>
     <row r="36" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="16" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="B36" s="25" t="s">
         <v>71</v>
@@ -3191,7 +3182,7 @@
     </row>
     <row r="41" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="16" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="B41" s="10" t="s">
         <v>80</v>
@@ -3237,10 +3228,10 @@
     </row>
     <row r="43" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="16" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C43" s="33">
         <v>52600</v>
@@ -3265,7 +3256,7 @@
     </row>
     <row r="44" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="16" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="B44" s="10" t="s">
         <v>83</v>
@@ -3289,7 +3280,7 @@
     </row>
     <row r="45" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="16" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="B45" s="10" t="s">
         <v>84</v>
@@ -3411,7 +3402,7 @@
     </row>
     <row r="50" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="21" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="B50" s="34" t="s">
         <v>1</v>
@@ -3863,10 +3854,10 @@
     </row>
     <row r="65" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="16" t="s">
+        <v>269</v>
+      </c>
+      <c r="B65" s="39" t="s">
         <v>121</v>
-      </c>
-      <c r="B65" s="39" t="s">
-        <v>122</v>
       </c>
       <c r="C65" s="12">
         <v>340204</v>
@@ -3875,7 +3866,7 @@
         <v>14</v>
       </c>
       <c r="E65" s="13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F65" s="13" t="s">
         <v>4</v>
@@ -3891,10 +3882,10 @@
     </row>
     <row r="66" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="16" t="s">
-        <v>124</v>
+        <v>269</v>
       </c>
       <c r="B66" s="39" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C66" s="12">
         <v>174705</v>
@@ -3903,7 +3894,7 @@
         <v>12</v>
       </c>
       <c r="E66" s="13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F66" s="35" t="s">
         <v>4</v>
@@ -3918,11 +3909,11 @@
       <c r="L66" s="13"/>
     </row>
     <row r="67" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="40" t="s">
-        <v>125</v>
+      <c r="A67" s="16" t="s">
+        <v>269</v>
       </c>
       <c r="B67" s="39" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C67" s="31">
         <v>2500000</v>
@@ -3931,7 +3922,7 @@
         <v>106</v>
       </c>
       <c r="E67" s="13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F67" s="13" t="s">
         <v>4</v>
@@ -3948,18 +3939,18 @@
       <c r="L67" s="13"/>
     </row>
     <row r="68" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="40" t="s">
-        <v>127</v>
+      <c r="A68" s="16" t="s">
+        <v>269</v>
       </c>
       <c r="B68" s="39" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C68" s="30">
         <v>1000000</v>
       </c>
       <c r="D68" s="12"/>
       <c r="E68" s="13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F68" s="13" t="s">
         <v>4</v>
@@ -3976,11 +3967,11 @@
       <c r="L68" s="13"/>
     </row>
     <row r="69" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="40" t="s">
-        <v>129</v>
+      <c r="A69" s="16" t="s">
+        <v>269</v>
       </c>
       <c r="B69" s="39" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C69" s="29">
         <v>139929</v>
@@ -3989,7 +3980,7 @@
         <v>27</v>
       </c>
       <c r="E69" s="13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F69" s="13" t="s">
         <v>4</v>
@@ -4007,17 +3998,17 @@
     </row>
     <row r="70" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="40" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B70" s="39" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="C70" s="30">
         <v>250000</v>
       </c>
       <c r="D70" s="12"/>
       <c r="E70" s="13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F70" s="13" t="s">
         <v>4</v>
@@ -4035,10 +4026,10 @@
     </row>
     <row r="71" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="16" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B71" s="39" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="C71" s="12">
         <v>2821906</v>
@@ -4047,7 +4038,7 @@
         <v>50</v>
       </c>
       <c r="E71" s="13" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F71" s="19" t="s">
         <v>4</v>
@@ -4061,17 +4052,17 @@
     </row>
     <row r="72" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="16" t="s">
-        <v>136</v>
+        <v>268</v>
       </c>
       <c r="B72" s="39" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C72" s="12"/>
       <c r="D72" s="12">
         <v>35</v>
       </c>
       <c r="E72" s="13" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F72" s="13" t="s">
         <v>4</v>
@@ -4087,10 +4078,10 @@
     </row>
     <row r="73" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="14" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="B73" s="41" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C73" s="12">
         <v>571838</v>
@@ -4099,7 +4090,7 @@
         <v>14</v>
       </c>
       <c r="E73" s="13" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="F73" s="13" t="s">
         <v>4</v>
@@ -4117,10 +4108,10 @@
     </row>
     <row r="74" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="16" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="B74" s="34" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C74" s="12">
         <v>4285981</v>
@@ -4149,10 +4140,10 @@
     </row>
     <row r="75" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="16" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="B75" s="24" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="C75" s="12">
         <v>705672</v>
@@ -4177,10 +4168,10 @@
     </row>
     <row r="76" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="16" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="B76" s="39" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C76" s="12">
         <v>121807</v>
@@ -4189,7 +4180,7 @@
         <v>5</v>
       </c>
       <c r="E76" s="13" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="F76" s="13" t="s">
         <v>4</v>
@@ -4207,10 +4198,10 @@
     </row>
     <row r="77" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="16" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="B77" s="39" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="C77" s="12">
         <v>621133</v>
@@ -4219,10 +4210,10 @@
         <v>22</v>
       </c>
       <c r="E77" s="13" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="F77" s="13" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="G77" s="13"/>
       <c r="H77" s="13" t="s">
@@ -4234,15 +4225,15 @@
         <v>4</v>
       </c>
       <c r="L77" s="13" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
     </row>
     <row r="78" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="16" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="B78" s="34" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C78" s="12">
         <v>267813</v>
@@ -4251,7 +4242,7 @@
         <v>20</v>
       </c>
       <c r="E78" s="38" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="F78" s="13" t="s">
         <v>3</v>
@@ -4269,10 +4260,10 @@
     </row>
     <row r="79" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="17" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B79" s="34" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="C79" s="15">
         <v>896000</v>
@@ -4281,7 +4272,7 @@
         <v>15</v>
       </c>
       <c r="E79" s="13" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="F79" s="13" t="s">
         <v>3</v>
@@ -4299,10 +4290,10 @@
     </row>
     <row r="80" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="14" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="B80" s="34" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C80" s="12">
         <v>60000</v>
@@ -4325,10 +4316,10 @@
     </row>
     <row r="81" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="16" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="B81" s="34" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="C81" s="15">
         <v>998871</v>
@@ -4337,10 +4328,10 @@
         <v>20</v>
       </c>
       <c r="E81" s="13" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="F81" s="13" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="G81" s="13"/>
       <c r="H81" s="13" t="s">
@@ -4359,10 +4350,10 @@
     </row>
     <row r="82" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="16" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="B82" s="39" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="C82" s="12">
         <v>993168</v>
@@ -4371,7 +4362,7 @@
         <v>27</v>
       </c>
       <c r="E82" s="13" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="F82" s="13" t="s">
         <v>95</v>
@@ -4391,10 +4382,10 @@
     </row>
     <row r="83" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="16" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B83" s="34" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C83" s="12">
         <v>615809</v>
@@ -4403,7 +4394,7 @@
         <v>19</v>
       </c>
       <c r="E83" s="13" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="F83" s="13" t="s">
         <v>95</v>
@@ -4425,10 +4416,10 @@
     </row>
     <row r="84" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="16" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="B84" s="34" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C84" s="15">
         <v>112288</v>
@@ -4453,17 +4444,17 @@
     </row>
     <row r="85" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="16" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B85" s="39" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="C85" s="12"/>
       <c r="D85" s="12">
         <v>112</v>
       </c>
       <c r="E85" s="13" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F85" s="13" t="s">
         <v>4</v>
@@ -4481,17 +4472,17 @@
     </row>
     <row r="86" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="16" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="B86" s="39" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C86" s="12"/>
       <c r="D86" s="12">
         <v>0</v>
       </c>
       <c r="E86" s="13" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F86" s="13" t="s">
         <v>4</v>
@@ -4509,17 +4500,17 @@
     </row>
     <row r="87" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="16" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="B87" s="39" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C87" s="12"/>
       <c r="D87" s="12">
         <v>0</v>
       </c>
       <c r="E87" s="13" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F87" s="13" t="s">
         <v>4</v>
@@ -4537,10 +4528,10 @@
     </row>
     <row r="88" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="16" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="B88" s="34" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="C88" s="43">
         <v>396396</v>
@@ -4549,7 +4540,7 @@
         <v>39</v>
       </c>
       <c r="E88" s="13" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F88" s="13" t="s">
         <v>4</v>
@@ -4569,15 +4560,15 @@
     </row>
     <row r="89" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="16" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B89" s="39" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="C89" s="12"/>
       <c r="D89" s="12"/>
       <c r="E89" s="13" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F89" s="13" t="s">
         <v>4</v>
@@ -4591,10 +4582,10 @@
     </row>
     <row r="90" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="16" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="B90" s="34" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="C90" s="12">
         <v>550000</v>
@@ -4603,7 +4594,7 @@
         <v>7</v>
       </c>
       <c r="E90" s="13" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="F90" s="13" t="s">
         <v>4</v>
@@ -4625,10 +4616,10 @@
     </row>
     <row r="91" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="16" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="B91" s="39" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="C91" s="12">
         <v>23877</v>
@@ -4637,7 +4628,7 @@
         <v>2</v>
       </c>
       <c r="E91" s="13" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F91" s="13" t="s">
         <v>4</v>
@@ -4653,10 +4644,10 @@
     </row>
     <row r="92" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="16" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="B92" s="39" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="C92" s="12"/>
       <c r="D92" s="12" t="e">
@@ -4664,7 +4655,7 @@
         <v>#REF!</v>
       </c>
       <c r="E92" s="13" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="F92" s="13" t="s">
         <v>4</v>
@@ -4678,13 +4669,13 @@
     </row>
     <row r="93" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="21" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B93" s="39"/>
       <c r="C93" s="12"/>
       <c r="D93" s="12"/>
       <c r="E93" s="13" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="F93" s="13" t="s">
         <v>4</v>
@@ -4698,17 +4689,17 @@
     </row>
     <row r="94" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="16" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="B94" s="39" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="C94" s="15">
         <v>550000</v>
       </c>
       <c r="D94" s="12"/>
       <c r="E94" s="13" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F94" s="13" t="s">
         <v>4</v>
@@ -4722,10 +4713,10 @@
     </row>
     <row r="95" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="16" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="B95" s="34" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C95" s="12">
         <v>282656</v>
@@ -4734,7 +4725,7 @@
         <v>12</v>
       </c>
       <c r="E95" s="13" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F95" s="13" t="s">
         <v>4</v>
@@ -4752,10 +4743,10 @@
     </row>
     <row r="96" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="16" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="B96" s="39" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="C96" s="12">
         <v>1259965</v>
@@ -4764,7 +4755,7 @@
         <v>27</v>
       </c>
       <c r="E96" s="13" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F96" s="13"/>
       <c r="G96" s="13"/>
@@ -4776,10 +4767,10 @@
     </row>
     <row r="97" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="16" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="B97" s="39" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="C97" s="12">
         <v>817999</v>
@@ -4808,10 +4799,10 @@
     </row>
     <row r="98" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="44" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B98" s="39" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="C98" s="45">
         <v>850000</v>
@@ -4820,7 +4811,7 @@
         <v>22</v>
       </c>
       <c r="E98" s="13" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="F98" s="13" t="s">
         <v>3</v>
@@ -4838,10 +4829,10 @@
     </row>
     <row r="99" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="21" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="B99" s="39" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="C99" s="12">
         <v>445964</v>
@@ -4850,7 +4841,7 @@
         <v>6</v>
       </c>
       <c r="E99" s="13" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="F99" s="13" t="s">
         <v>4</v>
@@ -4870,10 +4861,10 @@
     </row>
     <row r="100" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="21" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="B100" s="34" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="C100" s="12">
         <v>871045</v>
@@ -4885,11 +4876,11 @@
         <v>23</v>
       </c>
       <c r="F100" s="46" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="G100" s="13"/>
       <c r="H100" s="13" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="I100" s="13" t="s">
         <v>3</v>
@@ -4902,10 +4893,10 @@
     </row>
     <row r="101" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="21" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B101" s="34" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="C101" s="47"/>
       <c r="D101" s="13">
@@ -4932,17 +4923,17 @@
     </row>
     <row r="102" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="16" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="B102" s="34" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="C102" s="47"/>
       <c r="D102" s="13">
         <v>42</v>
       </c>
       <c r="E102" s="13" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="F102" s="13" t="s">
         <v>4</v>
@@ -4962,17 +4953,17 @@
     </row>
     <row r="103" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="16" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="B103" s="34" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="C103" s="47"/>
       <c r="D103" s="13">
         <v>136</v>
       </c>
       <c r="E103" s="13" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="F103" s="13" t="s">
         <v>4</v>
@@ -4998,10 +4989,10 @@
     </row>
     <row r="104" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="16" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="B104" s="39" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="C104" s="47">
         <v>175000</v>
@@ -5010,7 +5001,7 @@
         <v>10</v>
       </c>
       <c r="E104" s="13" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="F104" s="13" t="s">
         <v>4</v>
@@ -5032,7 +5023,7 @@
     </row>
     <row r="105" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="16" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="B105" s="39"/>
       <c r="C105" s="47">
@@ -5042,7 +5033,7 @@
         <v>10</v>
       </c>
       <c r="E105" s="13" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="F105" s="13"/>
       <c r="G105" s="13" t="s">
@@ -5062,19 +5053,19 @@
     </row>
     <row r="106" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="21" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="B106" s="39" t="s">
-        <v>222</v>
-      </c>
-      <c r="C106" s="47">
-        <v>300000</v>
+        <v>216</v>
+      </c>
+      <c r="C106" s="47" t="s">
+        <v>267</v>
       </c>
       <c r="D106" s="13">
         <v>78</v>
       </c>
       <c r="E106" s="13" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="F106" s="13"/>
       <c r="G106" s="13"/>
@@ -5092,23 +5083,23 @@
     </row>
     <row r="107" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="21" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="B107" s="39" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C107" s="13"/>
       <c r="D107" s="13">
         <v>72</v>
       </c>
       <c r="E107" s="13" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F107" s="13" t="s">
         <v>4</v>
       </c>
       <c r="G107" s="13" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="H107" s="13" t="s">
         <v>3</v>
@@ -5124,10 +5115,10 @@
     </row>
     <row r="108" spans="1:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="49" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="B108" s="39" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="C108" s="13">
         <v>372680</v>
@@ -5152,10 +5143,10 @@
     </row>
     <row r="109" spans="1:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="49" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="B109" s="34" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C109" s="47">
         <v>167000</v>
@@ -5164,10 +5155,10 @@
         <v>15</v>
       </c>
       <c r="E109" s="13" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="F109" s="13" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="G109" s="13" t="s">
         <v>3</v>
@@ -5188,10 +5179,10 @@
     </row>
     <row r="110" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="48" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B110" s="34" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="C110" s="47">
         <v>69129</v>
@@ -5220,7 +5211,7 @@
     </row>
     <row r="111" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="51" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="B111" s="34" t="s">
         <v>1</v>
@@ -5248,10 +5239,10 @@
     </row>
     <row r="112" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="51" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="B112" s="34" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="C112" s="50">
         <v>1000000</v>
@@ -5271,15 +5262,15 @@
       <c r="J112" s="50"/>
       <c r="K112" s="50"/>
       <c r="L112" s="50" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
     </row>
     <row r="113" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="51" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="B113" s="39" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="C113" s="50">
         <v>475000</v>
@@ -5288,7 +5279,7 @@
         <v>30</v>
       </c>
       <c r="E113" s="13" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="F113" s="50"/>
       <c r="G113" s="50" t="s">
@@ -5301,15 +5292,15 @@
       <c r="J113" s="50"/>
       <c r="K113" s="50"/>
       <c r="L113" s="50" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
     </row>
     <row r="114" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="51" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="B114" s="34" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="C114" s="50">
         <v>1140000</v>
@@ -5327,12 +5318,12 @@
       <c r="J114" s="50"/>
       <c r="K114" s="50"/>
       <c r="L114" s="50" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
     </row>
     <row r="115" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="49" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B115" s="52" t="s">
         <v>1</v>
@@ -5344,7 +5335,7 @@
         <v>15</v>
       </c>
       <c r="E115" s="13" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="F115" s="50"/>
       <c r="G115" s="50"/>
@@ -5358,10 +5349,10 @@
     </row>
     <row r="116" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="49" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="B116" s="54" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="C116" s="53">
         <v>1530000</v>
@@ -5370,7 +5361,7 @@
         <v>20</v>
       </c>
       <c r="E116" s="13" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="F116" s="50"/>
       <c r="G116" s="50"/>
@@ -5387,7 +5378,7 @@
         <v>3</v>
       </c>
       <c r="L116" s="50" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
     </row>
     <row r="117" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>